<commit_message>
content(abc): add apple image to c0u1-fc-1 flashcard
First real lesson image, authored via the P3 import path (image column in
the course workbook). Persists across reseeds since git is the content
source of truth.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/courses/c0-abc-first-words.xlsx
+++ b/courses/c0-abc-first-words.xlsx
@@ -552,7 +552,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M52"/>
+  <dimension ref="A1:N52"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -594,6 +594,9 @@
       <c r="M1" t="str">
         <v>pair5</v>
       </c>
+      <c r="N1" t="str">
+        <v>image</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -620,6 +623,24 @@
       <c r="H2" t="str">
         <v>แอปเปิล</v>
       </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v>https://cdn.jsdelivr.net/gh/twitter/twemoji@14.0.2/assets/72x72/1f34e.png</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -646,6 +667,24 @@
       <c r="H3" t="str">
         <v>ลูกบอล</v>
       </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -672,6 +711,24 @@
       <c r="H4" t="str">
         <v>แมว</v>
       </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -698,6 +755,24 @@
       <c r="H5" t="str">
         <v>หมา</v>
       </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -724,6 +799,24 @@
       <c r="H6" t="str">
         <v>ไข่</v>
       </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -750,6 +843,24 @@
       <c r="H7" t="str">
         <v>ปลา</v>
       </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -776,6 +887,24 @@
       <c r="H8" t="str">
         <v>แพะ</v>
       </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -802,6 +931,24 @@
       <c r="H9" t="str">
         <v>หมวก</v>
       </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -828,6 +975,24 @@
       <c r="H10" t="str">
         <v>น้ำแข็ง</v>
       </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -854,6 +1019,24 @@
       <c r="H11" t="str">
         <v>แยม</v>
       </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -880,6 +1063,24 @@
       <c r="H12" t="str">
         <v>ว่าว</v>
       </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -906,6 +1107,24 @@
       <c r="H13" t="str">
         <v>สิงโต</v>
       </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -932,6 +1151,24 @@
       <c r="H14" t="str">
         <v>นม</v>
       </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -949,6 +1186,12 @@
       <c r="E15">
         <v>1</v>
       </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
       <c r="H15" t="str">
         <v>จับคู่ตัวอักษรกับคำ</v>
       </c>
@@ -966,6 +1209,9 @@
       </c>
       <c r="M15" t="str">
         <v>E|egg|ไข่</v>
+      </c>
+      <c r="N15" t="str">
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -993,6 +1239,24 @@
       <c r="H16" t="str">
         <v>จมูก</v>
       </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v/>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -1019,6 +1283,24 @@
       <c r="H17" t="str">
         <v>ส้ม</v>
       </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v/>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
+      <c r="M17" t="str">
+        <v/>
+      </c>
+      <c r="N17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -1045,6 +1327,24 @@
       <c r="H18" t="str">
         <v>ปากกา</v>
       </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
+        <v/>
+      </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
+      <c r="M18" t="str">
+        <v/>
+      </c>
+      <c r="N18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1071,6 +1371,24 @@
       <c r="H19" t="str">
         <v>ราชินี</v>
       </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v/>
+      </c>
+      <c r="L19" t="str">
+        <v/>
+      </c>
+      <c r="M19" t="str">
+        <v/>
+      </c>
+      <c r="N19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -1097,6 +1415,24 @@
       <c r="H20" t="str">
         <v>สีแดง</v>
       </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v/>
+      </c>
+      <c r="L20" t="str">
+        <v/>
+      </c>
+      <c r="M20" t="str">
+        <v/>
+      </c>
+      <c r="N20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1123,6 +1459,24 @@
       <c r="H21" t="str">
         <v>พระอาทิตย์</v>
       </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v/>
+      </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+      <c r="M21" t="str">
+        <v/>
+      </c>
+      <c r="N21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1149,6 +1503,24 @@
       <c r="H22" t="str">
         <v>ต้นไม้</v>
       </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v/>
+      </c>
+      <c r="L22" t="str">
+        <v/>
+      </c>
+      <c r="M22" t="str">
+        <v/>
+      </c>
+      <c r="N22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1175,6 +1547,24 @@
       <c r="H23" t="str">
         <v>ร่ม</v>
       </c>
+      <c r="I23" t="str">
+        <v/>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23" t="str">
+        <v/>
+      </c>
+      <c r="L23" t="str">
+        <v/>
+      </c>
+      <c r="M23" t="str">
+        <v/>
+      </c>
+      <c r="N23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1201,6 +1591,24 @@
       <c r="H24" t="str">
         <v>รถตู้</v>
       </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
+        <v/>
+      </c>
+      <c r="L24" t="str">
+        <v/>
+      </c>
+      <c r="M24" t="str">
+        <v/>
+      </c>
+      <c r="N24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1227,6 +1635,24 @@
       <c r="H25" t="str">
         <v>น้ำ</v>
       </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
+        <v/>
+      </c>
+      <c r="L25" t="str">
+        <v/>
+      </c>
+      <c r="M25" t="str">
+        <v/>
+      </c>
+      <c r="N25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1253,6 +1679,24 @@
       <c r="H26" t="str">
         <v>กล่อง</v>
       </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
+        <v/>
+      </c>
+      <c r="L26" t="str">
+        <v/>
+      </c>
+      <c r="M26" t="str">
+        <v/>
+      </c>
+      <c r="N26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1279,6 +1723,24 @@
       <c r="H27" t="str">
         <v>โยโย่</v>
       </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
+        <v/>
+      </c>
+      <c r="L27" t="str">
+        <v/>
+      </c>
+      <c r="M27" t="str">
+        <v/>
+      </c>
+      <c r="N27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1305,6 +1767,24 @@
       <c r="H28" t="str">
         <v>สวนสัตว์</v>
       </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+      <c r="K28" t="str">
+        <v/>
+      </c>
+      <c r="L28" t="str">
+        <v/>
+      </c>
+      <c r="M28" t="str">
+        <v/>
+      </c>
+      <c r="N28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1322,6 +1802,12 @@
       <c r="E29">
         <v>1</v>
       </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
       <c r="H29" t="str">
         <v>จับคู่ตัวอักษรกับคำ</v>
       </c>
@@ -1339,6 +1825,9 @@
       </c>
       <c r="M29" t="str">
         <v>S|sun|พระอาทิตย์</v>
+      </c>
+      <c r="N29" t="str">
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -1366,6 +1855,24 @@
       <c r="H30" t="str">
         <v>สีแดง</v>
       </c>
+      <c r="I30" t="str">
+        <v/>
+      </c>
+      <c r="J30" t="str">
+        <v/>
+      </c>
+      <c r="K30" t="str">
+        <v/>
+      </c>
+      <c r="L30" t="str">
+        <v/>
+      </c>
+      <c r="M30" t="str">
+        <v/>
+      </c>
+      <c r="N30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1392,6 +1899,24 @@
       <c r="H31" t="str">
         <v>สีน้ำเงิน</v>
       </c>
+      <c r="I31" t="str">
+        <v/>
+      </c>
+      <c r="J31" t="str">
+        <v/>
+      </c>
+      <c r="K31" t="str">
+        <v/>
+      </c>
+      <c r="L31" t="str">
+        <v/>
+      </c>
+      <c r="M31" t="str">
+        <v/>
+      </c>
+      <c r="N31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1418,6 +1943,24 @@
       <c r="H32" t="str">
         <v>สีเขียว</v>
       </c>
+      <c r="I32" t="str">
+        <v/>
+      </c>
+      <c r="J32" t="str">
+        <v/>
+      </c>
+      <c r="K32" t="str">
+        <v/>
+      </c>
+      <c r="L32" t="str">
+        <v/>
+      </c>
+      <c r="M32" t="str">
+        <v/>
+      </c>
+      <c r="N32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1444,6 +1987,24 @@
       <c r="H33" t="str">
         <v>สีเหลือง</v>
       </c>
+      <c r="I33" t="str">
+        <v/>
+      </c>
+      <c r="J33" t="str">
+        <v/>
+      </c>
+      <c r="K33" t="str">
+        <v/>
+      </c>
+      <c r="L33" t="str">
+        <v/>
+      </c>
+      <c r="M33" t="str">
+        <v/>
+      </c>
+      <c r="N33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1470,6 +2031,24 @@
       <c r="H34" t="str">
         <v>สีดำ</v>
       </c>
+      <c r="I34" t="str">
+        <v/>
+      </c>
+      <c r="J34" t="str">
+        <v/>
+      </c>
+      <c r="K34" t="str">
+        <v/>
+      </c>
+      <c r="L34" t="str">
+        <v/>
+      </c>
+      <c r="M34" t="str">
+        <v/>
+      </c>
+      <c r="N34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -1496,6 +2075,24 @@
       <c r="H35" t="str">
         <v>สีขาว</v>
       </c>
+      <c r="I35" t="str">
+        <v/>
+      </c>
+      <c r="J35" t="str">
+        <v/>
+      </c>
+      <c r="K35" t="str">
+        <v/>
+      </c>
+      <c r="L35" t="str">
+        <v/>
+      </c>
+      <c r="M35" t="str">
+        <v/>
+      </c>
+      <c r="N35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -1513,6 +2110,12 @@
       <c r="E36">
         <v>1</v>
       </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
       <c r="H36" t="str">
         <v>จับคู่สีกับคำไทย</v>
       </c>
@@ -1530,6 +2133,9 @@
       </c>
       <c r="M36" t="str">
         <v>black|ดำ|สีดำ</v>
+      </c>
+      <c r="N36" t="str">
+        <v/>
       </c>
     </row>
     <row r="37">
@@ -1557,6 +2163,24 @@
       <c r="H37" t="str">
         <v>สวัสดี</v>
       </c>
+      <c r="I37" t="str">
+        <v/>
+      </c>
+      <c r="J37" t="str">
+        <v/>
+      </c>
+      <c r="K37" t="str">
+        <v/>
+      </c>
+      <c r="L37" t="str">
+        <v/>
+      </c>
+      <c r="M37" t="str">
+        <v/>
+      </c>
+      <c r="N37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -1583,6 +2207,24 @@
       <c r="H38" t="str">
         <v>หวัดดี</v>
       </c>
+      <c r="I38" t="str">
+        <v/>
+      </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
+      <c r="K38" t="str">
+        <v/>
+      </c>
+      <c r="L38" t="str">
+        <v/>
+      </c>
+      <c r="M38" t="str">
+        <v/>
+      </c>
+      <c r="N38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -1609,6 +2251,24 @@
       <c r="H39" t="str">
         <v>ลาก่อน</v>
       </c>
+      <c r="I39" t="str">
+        <v/>
+      </c>
+      <c r="J39" t="str">
+        <v/>
+      </c>
+      <c r="K39" t="str">
+        <v/>
+      </c>
+      <c r="L39" t="str">
+        <v/>
+      </c>
+      <c r="M39" t="str">
+        <v/>
+      </c>
+      <c r="N39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -1635,6 +2295,24 @@
       <c r="H40" t="str">
         <v>ใช่</v>
       </c>
+      <c r="I40" t="str">
+        <v/>
+      </c>
+      <c r="J40" t="str">
+        <v/>
+      </c>
+      <c r="K40" t="str">
+        <v/>
+      </c>
+      <c r="L40" t="str">
+        <v/>
+      </c>
+      <c r="M40" t="str">
+        <v/>
+      </c>
+      <c r="N40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -1661,6 +2339,24 @@
       <c r="H41" t="str">
         <v>ไม่</v>
       </c>
+      <c r="I41" t="str">
+        <v/>
+      </c>
+      <c r="J41" t="str">
+        <v/>
+      </c>
+      <c r="K41" t="str">
+        <v/>
+      </c>
+      <c r="L41" t="str">
+        <v/>
+      </c>
+      <c r="M41" t="str">
+        <v/>
+      </c>
+      <c r="N41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -1687,6 +2383,24 @@
       <c r="H42" t="str">
         <v>กรุณา</v>
       </c>
+      <c r="I42" t="str">
+        <v/>
+      </c>
+      <c r="J42" t="str">
+        <v/>
+      </c>
+      <c r="K42" t="str">
+        <v/>
+      </c>
+      <c r="L42" t="str">
+        <v/>
+      </c>
+      <c r="M42" t="str">
+        <v/>
+      </c>
+      <c r="N42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -1713,6 +2427,24 @@
       <c r="H43" t="str">
         <v>ขอบคุณ</v>
       </c>
+      <c r="I43" t="str">
+        <v/>
+      </c>
+      <c r="J43" t="str">
+        <v/>
+      </c>
+      <c r="K43" t="str">
+        <v/>
+      </c>
+      <c r="L43" t="str">
+        <v/>
+      </c>
+      <c r="M43" t="str">
+        <v/>
+      </c>
+      <c r="N43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -1730,6 +2462,12 @@
       <c r="E44">
         <v>1</v>
       </c>
+      <c r="F44" t="str">
+        <v/>
+      </c>
+      <c r="G44" t="str">
+        <v/>
+      </c>
       <c r="H44" t="str">
         <v>จับคู่คำทักทายกับคำไทย</v>
       </c>
@@ -1747,6 +2485,9 @@
       </c>
       <c r="M44" t="str">
         <v>thank you|ขอบคุณ|ขอบคุณ</v>
+      </c>
+      <c r="N44" t="str">
+        <v/>
       </c>
     </row>
     <row r="45">
@@ -1774,6 +2515,24 @@
       <c r="H45" t="str">
         <v>หนังสือ</v>
       </c>
+      <c r="I45" t="str">
+        <v/>
+      </c>
+      <c r="J45" t="str">
+        <v/>
+      </c>
+      <c r="K45" t="str">
+        <v/>
+      </c>
+      <c r="L45" t="str">
+        <v/>
+      </c>
+      <c r="M45" t="str">
+        <v/>
+      </c>
+      <c r="N45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -1800,6 +2559,24 @@
       <c r="H46" t="str">
         <v>ปากกา</v>
       </c>
+      <c r="I46" t="str">
+        <v/>
+      </c>
+      <c r="J46" t="str">
+        <v/>
+      </c>
+      <c r="K46" t="str">
+        <v/>
+      </c>
+      <c r="L46" t="str">
+        <v/>
+      </c>
+      <c r="M46" t="str">
+        <v/>
+      </c>
+      <c r="N46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -1826,6 +2603,24 @@
       <c r="H47" t="str">
         <v>ดินสอ</v>
       </c>
+      <c r="I47" t="str">
+        <v/>
+      </c>
+      <c r="J47" t="str">
+        <v/>
+      </c>
+      <c r="K47" t="str">
+        <v/>
+      </c>
+      <c r="L47" t="str">
+        <v/>
+      </c>
+      <c r="M47" t="str">
+        <v/>
+      </c>
+      <c r="N47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -1852,6 +2647,24 @@
       <c r="H48" t="str">
         <v>โต๊ะ</v>
       </c>
+      <c r="I48" t="str">
+        <v/>
+      </c>
+      <c r="J48" t="str">
+        <v/>
+      </c>
+      <c r="K48" t="str">
+        <v/>
+      </c>
+      <c r="L48" t="str">
+        <v/>
+      </c>
+      <c r="M48" t="str">
+        <v/>
+      </c>
+      <c r="N48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -1878,6 +2691,24 @@
       <c r="H49" t="str">
         <v>กระเป๋า</v>
       </c>
+      <c r="I49" t="str">
+        <v/>
+      </c>
+      <c r="J49" t="str">
+        <v/>
+      </c>
+      <c r="K49" t="str">
+        <v/>
+      </c>
+      <c r="L49" t="str">
+        <v/>
+      </c>
+      <c r="M49" t="str">
+        <v/>
+      </c>
+      <c r="N49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -1904,6 +2735,24 @@
       <c r="H50" t="str">
         <v>ครู</v>
       </c>
+      <c r="I50" t="str">
+        <v/>
+      </c>
+      <c r="J50" t="str">
+        <v/>
+      </c>
+      <c r="K50" t="str">
+        <v/>
+      </c>
+      <c r="L50" t="str">
+        <v/>
+      </c>
+      <c r="M50" t="str">
+        <v/>
+      </c>
+      <c r="N50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -1930,6 +2779,24 @@
       <c r="H51" t="str">
         <v>นักเรียน</v>
       </c>
+      <c r="I51" t="str">
+        <v/>
+      </c>
+      <c r="J51" t="str">
+        <v/>
+      </c>
+      <c r="K51" t="str">
+        <v/>
+      </c>
+      <c r="L51" t="str">
+        <v/>
+      </c>
+      <c r="M51" t="str">
+        <v/>
+      </c>
+      <c r="N51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -1947,6 +2814,12 @@
       <c r="E52">
         <v>1</v>
       </c>
+      <c r="F52" t="str">
+        <v/>
+      </c>
+      <c r="G52" t="str">
+        <v/>
+      </c>
       <c r="H52" t="str">
         <v>จับคู่ของในห้องเรียนกับคำไทย</v>
       </c>
@@ -1965,10 +2838,13 @@
       <c r="M52" t="str">
         <v>bag|กระเป๋า|กระเป๋า</v>
       </c>
+      <c r="N52" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M52"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N52"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
content(abc): image ABC course with OpenMoji SVGs
Author self-hosted lesson images across the ABC & First Words course:
43 flashcards and 19 matching pairs now carry pictures. Assets are
OpenMoji SVGs (CC BY-SA 4.0) committed under public/img/lessons/ and
referenced by relative /img/lessons/<word>.svg paths, so they persist
via the git-as-source-of-truth content model and survive emulator
restarts (unlike Storage-emulator uploads, which are wiped each start).

Words with no clean/distinct emoji are left imageless (jam, zoo, desk);
u4 greetings get gesture images on flashcards but not on the matching
game, where identical gestures would defeat the match. Matching images
sit on the English-word side. The apple proof is moved off the external
twemoji CDN onto the local SVG for consistency.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/courses/c0-abc-first-words.xlsx
+++ b/courses/c0-abc-first-words.xlsx
@@ -639,7 +639,7 @@
         <v/>
       </c>
       <c r="N2" t="str">
-        <v>https://cdn.jsdelivr.net/gh/twitter/twemoji@14.0.2/assets/72x72/1f34e.png</v>
+        <v>/img/lessons/apple.svg</v>
       </c>
     </row>
     <row r="3">
@@ -683,7 +683,7 @@
         <v/>
       </c>
       <c r="N3" t="str">
-        <v/>
+        <v>/img/lessons/ball.svg</v>
       </c>
     </row>
     <row r="4">
@@ -727,7 +727,7 @@
         <v/>
       </c>
       <c r="N4" t="str">
-        <v/>
+        <v>/img/lessons/cat.svg</v>
       </c>
     </row>
     <row r="5">
@@ -771,7 +771,7 @@
         <v/>
       </c>
       <c r="N5" t="str">
-        <v/>
+        <v>/img/lessons/dog.svg</v>
       </c>
     </row>
     <row r="6">
@@ -815,7 +815,7 @@
         <v/>
       </c>
       <c r="N6" t="str">
-        <v/>
+        <v>/img/lessons/egg.svg</v>
       </c>
     </row>
     <row r="7">
@@ -859,7 +859,7 @@
         <v/>
       </c>
       <c r="N7" t="str">
-        <v/>
+        <v>/img/lessons/fish.svg</v>
       </c>
     </row>
     <row r="8">
@@ -903,7 +903,7 @@
         <v/>
       </c>
       <c r="N8" t="str">
-        <v/>
+        <v>/img/lessons/goat.svg</v>
       </c>
     </row>
     <row r="9">
@@ -947,7 +947,7 @@
         <v/>
       </c>
       <c r="N9" t="str">
-        <v/>
+        <v>/img/lessons/hat.svg</v>
       </c>
     </row>
     <row r="10">
@@ -991,7 +991,7 @@
         <v/>
       </c>
       <c r="N10" t="str">
-        <v/>
+        <v>/img/lessons/ice.svg</v>
       </c>
     </row>
     <row r="11">
@@ -1079,7 +1079,7 @@
         <v/>
       </c>
       <c r="N12" t="str">
-        <v/>
+        <v>/img/lessons/kite.svg</v>
       </c>
     </row>
     <row r="13">
@@ -1123,7 +1123,7 @@
         <v/>
       </c>
       <c r="N13" t="str">
-        <v/>
+        <v>/img/lessons/lion.svg</v>
       </c>
     </row>
     <row r="14">
@@ -1167,7 +1167,7 @@
         <v/>
       </c>
       <c r="N14" t="str">
-        <v/>
+        <v>/img/lessons/milk.svg</v>
       </c>
     </row>
     <row r="15">
@@ -1196,19 +1196,19 @@
         <v>จับคู่ตัวอักษรกับคำ</v>
       </c>
       <c r="I15" t="str">
-        <v>A|apple|แอปเปิล</v>
+        <v>A|apple|แอปเปิล|ri=/img/lessons/apple.svg</v>
       </c>
       <c r="J15" t="str">
-        <v>B|ball|ลูกบอล</v>
+        <v>B|ball|ลูกบอล|ri=/img/lessons/ball.svg</v>
       </c>
       <c r="K15" t="str">
-        <v>C|cat|แมว</v>
+        <v>C|cat|แมว|ri=/img/lessons/cat.svg</v>
       </c>
       <c r="L15" t="str">
-        <v>D|dog|หมา</v>
+        <v>D|dog|หมา|ri=/img/lessons/dog.svg</v>
       </c>
       <c r="M15" t="str">
-        <v>E|egg|ไข่</v>
+        <v>E|egg|ไข่|ri=/img/lessons/egg.svg</v>
       </c>
       <c r="N15" t="str">
         <v/>
@@ -1255,7 +1255,7 @@
         <v/>
       </c>
       <c r="N16" t="str">
-        <v/>
+        <v>/img/lessons/nose.svg</v>
       </c>
     </row>
     <row r="17">
@@ -1299,7 +1299,7 @@
         <v/>
       </c>
       <c r="N17" t="str">
-        <v/>
+        <v>/img/lessons/orange.svg</v>
       </c>
     </row>
     <row r="18">
@@ -1343,7 +1343,7 @@
         <v/>
       </c>
       <c r="N18" t="str">
-        <v/>
+        <v>/img/lessons/pen.svg</v>
       </c>
     </row>
     <row r="19">
@@ -1387,7 +1387,7 @@
         <v/>
       </c>
       <c r="N19" t="str">
-        <v/>
+        <v>/img/lessons/queen.svg</v>
       </c>
     </row>
     <row r="20">
@@ -1431,7 +1431,7 @@
         <v/>
       </c>
       <c r="N20" t="str">
-        <v/>
+        <v>/img/lessons/red.svg</v>
       </c>
     </row>
     <row r="21">
@@ -1475,7 +1475,7 @@
         <v/>
       </c>
       <c r="N21" t="str">
-        <v/>
+        <v>/img/lessons/sun.svg</v>
       </c>
     </row>
     <row r="22">
@@ -1519,7 +1519,7 @@
         <v/>
       </c>
       <c r="N22" t="str">
-        <v/>
+        <v>/img/lessons/tree.svg</v>
       </c>
     </row>
     <row r="23">
@@ -1563,7 +1563,7 @@
         <v/>
       </c>
       <c r="N23" t="str">
-        <v/>
+        <v>/img/lessons/umbrella.svg</v>
       </c>
     </row>
     <row r="24">
@@ -1607,7 +1607,7 @@
         <v/>
       </c>
       <c r="N24" t="str">
-        <v/>
+        <v>/img/lessons/van.svg</v>
       </c>
     </row>
     <row r="25">
@@ -1651,7 +1651,7 @@
         <v/>
       </c>
       <c r="N25" t="str">
-        <v/>
+        <v>/img/lessons/water.svg</v>
       </c>
     </row>
     <row r="26">
@@ -1695,7 +1695,7 @@
         <v/>
       </c>
       <c r="N26" t="str">
-        <v/>
+        <v>/img/lessons/box.svg</v>
       </c>
     </row>
     <row r="27">
@@ -1739,7 +1739,7 @@
         <v/>
       </c>
       <c r="N27" t="str">
-        <v/>
+        <v>/img/lessons/yoyo.svg</v>
       </c>
     </row>
     <row r="28">
@@ -1812,19 +1812,19 @@
         <v>จับคู่ตัวอักษรกับคำ</v>
       </c>
       <c r="I29" t="str">
-        <v>N|nose|จมูก</v>
+        <v>N|nose|จมูก|ri=/img/lessons/nose.svg</v>
       </c>
       <c r="J29" t="str">
-        <v>O|orange|ส้ม</v>
+        <v>O|orange|ส้ม|ri=/img/lessons/orange.svg</v>
       </c>
       <c r="K29" t="str">
-        <v>P|pen|ปากกา</v>
+        <v>P|pen|ปากกา|ri=/img/lessons/pen.svg</v>
       </c>
       <c r="L29" t="str">
-        <v>Q|queen|ราชินี</v>
+        <v>Q|queen|ราชินี|ri=/img/lessons/queen.svg</v>
       </c>
       <c r="M29" t="str">
-        <v>S|sun|พระอาทิตย์</v>
+        <v>S|sun|พระอาทิตย์|ri=/img/lessons/sun.svg</v>
       </c>
       <c r="N29" t="str">
         <v/>
@@ -1871,7 +1871,7 @@
         <v/>
       </c>
       <c r="N30" t="str">
-        <v/>
+        <v>/img/lessons/red.svg</v>
       </c>
     </row>
     <row r="31">
@@ -1915,7 +1915,7 @@
         <v/>
       </c>
       <c r="N31" t="str">
-        <v/>
+        <v>/img/lessons/blue.svg</v>
       </c>
     </row>
     <row r="32">
@@ -1959,7 +1959,7 @@
         <v/>
       </c>
       <c r="N32" t="str">
-        <v/>
+        <v>/img/lessons/green.svg</v>
       </c>
     </row>
     <row r="33">
@@ -2003,7 +2003,7 @@
         <v/>
       </c>
       <c r="N33" t="str">
-        <v/>
+        <v>/img/lessons/yellow.svg</v>
       </c>
     </row>
     <row r="34">
@@ -2047,7 +2047,7 @@
         <v/>
       </c>
       <c r="N34" t="str">
-        <v/>
+        <v>/img/lessons/black.svg</v>
       </c>
     </row>
     <row r="35">
@@ -2091,7 +2091,7 @@
         <v/>
       </c>
       <c r="N35" t="str">
-        <v/>
+        <v>/img/lessons/white.svg</v>
       </c>
     </row>
     <row r="36">
@@ -2120,19 +2120,19 @@
         <v>จับคู่สีกับคำไทย</v>
       </c>
       <c r="I36" t="str">
-        <v>red|แดง|สีแดง</v>
+        <v>red|แดง|สีแดง|li=/img/lessons/red.svg</v>
       </c>
       <c r="J36" t="str">
-        <v>blue|น้ำเงิน|สีน้ำเงิน</v>
+        <v>blue|น้ำเงิน|สีน้ำเงิน|li=/img/lessons/blue.svg</v>
       </c>
       <c r="K36" t="str">
-        <v>green|เขียว|สีเขียว</v>
+        <v>green|เขียว|สีเขียว|li=/img/lessons/green.svg</v>
       </c>
       <c r="L36" t="str">
-        <v>yellow|เหลือง|สีเหลือง</v>
+        <v>yellow|เหลือง|สีเหลือง|li=/img/lessons/yellow.svg</v>
       </c>
       <c r="M36" t="str">
-        <v>black|ดำ|สีดำ</v>
+        <v>black|ดำ|สีดำ|li=/img/lessons/black.svg</v>
       </c>
       <c r="N36" t="str">
         <v/>
@@ -2179,7 +2179,7 @@
         <v/>
       </c>
       <c r="N37" t="str">
-        <v/>
+        <v>/img/lessons/wave.svg</v>
       </c>
     </row>
     <row r="38">
@@ -2223,7 +2223,7 @@
         <v/>
       </c>
       <c r="N38" t="str">
-        <v/>
+        <v>/img/lessons/wave.svg</v>
       </c>
     </row>
     <row r="39">
@@ -2267,7 +2267,7 @@
         <v/>
       </c>
       <c r="N39" t="str">
-        <v/>
+        <v>/img/lessons/wave.svg</v>
       </c>
     </row>
     <row r="40">
@@ -2311,7 +2311,7 @@
         <v/>
       </c>
       <c r="N40" t="str">
-        <v/>
+        <v>/img/lessons/thumbsup.svg</v>
       </c>
     </row>
     <row r="41">
@@ -2355,7 +2355,7 @@
         <v/>
       </c>
       <c r="N41" t="str">
-        <v/>
+        <v>/img/lessons/thumbsdown.svg</v>
       </c>
     </row>
     <row r="42">
@@ -2399,7 +2399,7 @@
         <v/>
       </c>
       <c r="N42" t="str">
-        <v/>
+        <v>/img/lessons/pray.svg</v>
       </c>
     </row>
     <row r="43">
@@ -2443,7 +2443,7 @@
         <v/>
       </c>
       <c r="N43" t="str">
-        <v/>
+        <v>/img/lessons/pray.svg</v>
       </c>
     </row>
     <row r="44">
@@ -2531,7 +2531,7 @@
         <v/>
       </c>
       <c r="N45" t="str">
-        <v/>
+        <v>/img/lessons/book.svg</v>
       </c>
     </row>
     <row r="46">
@@ -2575,7 +2575,7 @@
         <v/>
       </c>
       <c r="N46" t="str">
-        <v/>
+        <v>/img/lessons/pen.svg</v>
       </c>
     </row>
     <row r="47">
@@ -2619,7 +2619,7 @@
         <v/>
       </c>
       <c r="N47" t="str">
-        <v/>
+        <v>/img/lessons/pencil.svg</v>
       </c>
     </row>
     <row r="48">
@@ -2707,7 +2707,7 @@
         <v/>
       </c>
       <c r="N49" t="str">
-        <v/>
+        <v>/img/lessons/bag.svg</v>
       </c>
     </row>
     <row r="50">
@@ -2751,7 +2751,7 @@
         <v/>
       </c>
       <c r="N50" t="str">
-        <v/>
+        <v>/img/lessons/teacher.svg</v>
       </c>
     </row>
     <row r="51">
@@ -2795,7 +2795,7 @@
         <v/>
       </c>
       <c r="N51" t="str">
-        <v/>
+        <v>/img/lessons/student.svg</v>
       </c>
     </row>
     <row r="52">
@@ -2824,19 +2824,19 @@
         <v>จับคู่ของในห้องเรียนกับคำไทย</v>
       </c>
       <c r="I52" t="str">
-        <v>book|หนังสือ|หนังสือ</v>
+        <v>book|หนังสือ|หนังสือ|li=/img/lessons/book.svg</v>
       </c>
       <c r="J52" t="str">
-        <v>pen|ปากกา|ปากกา</v>
+        <v>pen|ปากกา|ปากกา|li=/img/lessons/pen.svg</v>
       </c>
       <c r="K52" t="str">
-        <v>pencil|ดินสอ|ดินสอ</v>
+        <v>pencil|ดินสอ|ดินสอ|li=/img/lessons/pencil.svg</v>
       </c>
       <c r="L52" t="str">
         <v>desk|โต๊ะ|โต๊ะ</v>
       </c>
       <c r="M52" t="str">
-        <v>bag|กระเป๋า|กระเป๋า</v>
+        <v>bag|กระเป๋า|กระเป๋า|li=/img/lessons/bag.svg</v>
       </c>
       <c r="N52" t="str">
         <v/>

</xml_diff>